<commit_message>
P0 XLSX fixes · Exit P&L% + Position ID + Alerts wiring (external audit)
External audit PDF caught 4 P0 bugs in aegis_history.xlsx that my own
analysis missed. Verified empirically then fixed:

- Exit P&L% = 0 for all 52 rotation exits → backfill now computes from
  Current Perf when Status=EXIT · 52/52 → 6/52 remaining (delisted tix)
- Position ID populated 71/224 → 245/280 via always-populate in row output
  + backfill for historical rows
- Alerts column 0/224 → 11/280 via _load_alert_with_fallback wiring
  position_store-derived STOP_LOSS_HIT / DEEP_LOSS / RAPID_APPRECIATION
  triggers (bypasses R006 wiring gap · still Sprint K+ item at engine layer)
- Lifecycle State constant 'NEW' → column dropped (redundant with Position
  Stage · was misleading operator)
- Turnover σ dead column (0/224) → dropped

Column count: 54 → 49. Single sheet preserved. Zero R1/R2 touches.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/telegram/aegis_daily_2026-08-06.xlsx
+++ b/reports/telegram/aegis_daily_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AEGIS Daily" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AEGIS Daily'!$A$1:$AX$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AEGIS Daily'!$A$1:$AW$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX72"/>
+  <dimension ref="A1:AW72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,7 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="50" customWidth="1" min="19" max="19"/>
     <col width="60" customWidth="1" min="20" max="20"/>
-    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="44" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -482,12 +482,11 @@
     <col width="15" customWidth="1" min="42" max="42"/>
     <col width="12" customWidth="1" min="43" max="43"/>
     <col width="11" customWidth="1" min="44" max="44"/>
-    <col width="16" customWidth="1" min="45" max="45"/>
-    <col width="32" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
-    <col width="18" customWidth="1" min="48" max="48"/>
-    <col width="17" customWidth="1" min="49" max="49"/>
-    <col width="20" customWidth="1" min="50" max="50"/>
+    <col width="32" customWidth="1" min="45" max="45"/>
+    <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="17" customWidth="1" min="48" max="48"/>
+    <col width="20" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -593,7 +592,7 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerts</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -713,30 +712,25 @@
       </c>
       <c r="AS1" s="1" t="inlineStr">
         <is>
-          <t>Lifecycle State</t>
+          <t>Top Drivers</t>
         </is>
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>Top Drivers</t>
+          <t>Sector</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
-          <t>Sector</t>
+          <t>Portfolio Weight %</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>Portfolio Weight %</t>
+          <t>Expected Alpha %</t>
         </is>
       </c>
       <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Alpha %</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>Last Updated (UTC)</t>
         </is>
@@ -745,7 +739,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TCS_IND_20260729</t>
+          <t>GNFC_IND_20260806</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -760,19 +754,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R2_NEW</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>TCS</t>
-        </is>
-      </c>
+          <t>GNFC</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
@@ -788,14 +778,10 @@
       <c r="K2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="M2" s="3" t="n">
-        <v>-8</v>
-      </c>
+      <c r="L2" s="3" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="3" t="n">
-        <v>75.90000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
@@ -808,7 +794,7 @@
         </is>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>38.6</v>
+        <v>33.3</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>-0.8</v>
@@ -820,12 +806,12 @@
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-1.0%) · Rank ↑ 9→1 · Conf 39% · band HOLD · 16d left · → STRONG BUY</t>
+          <t>🟢 BUY (Δ-1.0%) · Rank #1 · Conf 34% · band HOLD · 17d left · → STRONG BUY</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr"/>
       <c r="V2" s="3" t="n">
-        <v>39.3</v>
+        <v>34.1</v>
       </c>
       <c r="W2" s="3" t="inlineStr">
         <is>
@@ -833,97 +819,88 @@
         </is>
       </c>
       <c r="X2" s="3" t="n">
-        <v>28.4</v>
+        <v>32.8</v>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z2" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA2" s="3" t="n">
         <v>17</v>
       </c>
       <c r="AB2" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AC2" s="3" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="AD2" s="3" t="n">
-        <v>2421.9</v>
+        <v>553.3</v>
       </c>
       <c r="AE2" s="3" t="n">
-        <v>2452.2</v>
+        <v>553.2999877929688</v>
       </c>
       <c r="AF2" s="3" t="n">
-        <v>2397.68</v>
+        <v>547.77</v>
       </c>
       <c r="AG2" s="3" t="n">
-        <v>2446.12</v>
+        <v>558.83</v>
       </c>
       <c r="AH2" s="3" t="n">
-        <v>2276.59</v>
+        <v>520.1</v>
       </c>
       <c r="AI2" s="3" t="n">
-        <v>-7.16</v>
+        <v>-6</v>
       </c>
       <c r="AJ2" s="3" t="n">
-        <v>2712.53</v>
+        <v>619.7</v>
       </c>
       <c r="AK2" s="3" t="n">
-        <v>10.62</v>
+        <v>12</v>
       </c>
       <c r="AL2" s="3" t="n">
-        <v>3003.16</v>
+        <v>686.09</v>
       </c>
       <c r="AM2" s="3" t="n">
-        <v>22.47</v>
+        <v>24</v>
       </c>
       <c r="AN2" s="3" t="n">
-        <v>2460</v>
+        <v>519.75</v>
       </c>
       <c r="AO2" s="3" t="n">
-        <v>-1.55</v>
+        <v>6.46</v>
       </c>
       <c r="AP2" s="3" t="n">
-        <v>-1.24</v>
-      </c>
-      <c r="AQ2" s="3" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="AR2" s="3" t="n">
-        <v>-4.11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="3" t="inlineStr"/>
+      <c r="AR2" s="3" t="inlineStr"/>
       <c r="AS2" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT2" s="3" t="inlineStr">
-        <is>
-          <t>Quality · Mean Reversion · Ai Hybrid</t>
-        </is>
-      </c>
-      <c r="AU2" s="3" t="inlineStr"/>
+          <t>Value · Growth · Ai Hybrid</t>
+        </is>
+      </c>
+      <c r="AT2" s="3" t="inlineStr"/>
+      <c r="AU2" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV2" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AX2" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>OFSS_IND_20260730</t>
+          <t>TCS_IND_20260729</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -943,10 +920,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>OFSS</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>STRONG BUY</t>
@@ -963,13 +944,13 @@
         <v>2</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
@@ -982,7 +963,7 @@
         </is>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>45.6</v>
+        <v>38.6</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>-0.8</v>
@@ -994,12 +975,12 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-1.0%) · Rank ↑ 6→2 · Conf 46% · band HOLD · 16d left · → STRONG BUY</t>
+          <t>🟢 BUY (Δ-1.0%) · Rank ↑ 9→2 · Conf 39% · band HOLD · 16d left · → STRONG BUY</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr"/>
       <c r="V3" s="3" t="n">
-        <v>46.4</v>
+        <v>39.3</v>
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
@@ -1007,13 +988,13 @@
         </is>
       </c>
       <c r="X3" s="3" t="n">
-        <v>27.2</v>
+        <v>28.4</v>
       </c>
       <c r="Y3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="Z3" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA3" s="3" t="n">
         <v>17</v>
@@ -1023,81 +1004,76 @@
       </c>
       <c r="AC3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="AD3" s="3" t="n">
-        <v>11727</v>
+        <v>2421.9</v>
       </c>
       <c r="AE3" s="3" t="n">
-        <v>11427</v>
+        <v>2452.2</v>
       </c>
       <c r="AF3" s="3" t="n">
-        <v>11609.73</v>
+        <v>2397.68</v>
       </c>
       <c r="AG3" s="3" t="n">
-        <v>11844.27</v>
+        <v>2446.12</v>
       </c>
       <c r="AH3" s="3" t="n">
-        <v>11023.38</v>
+        <v>2276.59</v>
       </c>
       <c r="AI3" s="3" t="n">
-        <v>-3.53</v>
+        <v>-7.16</v>
       </c>
       <c r="AJ3" s="3" t="n">
-        <v>13134.24</v>
+        <v>2712.53</v>
       </c>
       <c r="AK3" s="3" t="n">
-        <v>14.94</v>
+        <v>10.62</v>
       </c>
       <c r="AL3" s="3" t="n">
-        <v>14541.48</v>
+        <v>3003.16</v>
       </c>
       <c r="AM3" s="3" t="n">
-        <v>27.26</v>
+        <v>22.47</v>
       </c>
       <c r="AN3" s="3" t="n">
-        <v>11600</v>
+        <v>2460</v>
       </c>
       <c r="AO3" s="3" t="n">
-        <v>1.09</v>
+        <v>-1.55</v>
       </c>
       <c r="AP3" s="3" t="n">
-        <v>2.63</v>
+        <v>-1.24</v>
       </c>
       <c r="AQ3" s="3" t="n">
-        <v>1.51</v>
+        <v>0.32</v>
       </c>
       <c r="AR3" s="3" t="n">
-        <v>-3.08</v>
+        <v>-4.11</v>
       </c>
       <c r="AS3" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT3" s="3" t="inlineStr">
-        <is>
-          <t>Quality · Growth · Momentum</t>
-        </is>
-      </c>
-      <c r="AU3" s="3" t="inlineStr"/>
+          <t>Quality · Mean Reversion · Ai Hybrid</t>
+        </is>
+      </c>
+      <c r="AT3" s="3" t="inlineStr"/>
+      <c r="AU3" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV3" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AX3" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>INDIANB_IND_20260806</t>
+          <t>OFSS_IND_20260730</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1117,7 +1093,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>INDIANB</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -1136,10 +1112,14 @@
       <c r="K4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>-3</v>
+      </c>
       <c r="N4" s="3" t="n">
-        <v>68.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
@@ -1152,7 +1132,7 @@
         </is>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>34.2</v>
+        <v>45.6</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>-0.8</v>
@@ -1164,12 +1144,12 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-1.0%) · Rank #3 · Conf 35% · band HOLD · 17d left · → BUY</t>
+          <t>🟢 BUY (Δ-1.0%) · Rank ↑ 6→3 · Conf 46% · band HOLD · 16d left · → BUY</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr"/>
       <c r="V4" s="3" t="n">
-        <v>35</v>
+        <v>46.4</v>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
@@ -1177,93 +1157,92 @@
         </is>
       </c>
       <c r="X4" s="3" t="n">
-        <v>25.4</v>
+        <v>27.1</v>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z4" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA4" s="3" t="n">
         <v>17</v>
       </c>
       <c r="AB4" s="3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="AD4" s="3" t="n">
-        <v>853.4</v>
+        <v>11727</v>
       </c>
       <c r="AE4" s="3" t="n">
-        <v>853.4000244140625</v>
+        <v>11427</v>
       </c>
       <c r="AF4" s="3" t="n">
-        <v>844.87</v>
+        <v>11609.73</v>
       </c>
       <c r="AG4" s="3" t="n">
-        <v>861.9299999999999</v>
+        <v>11844.27</v>
       </c>
       <c r="AH4" s="3" t="n">
-        <v>802.2</v>
+        <v>11023.38</v>
       </c>
       <c r="AI4" s="3" t="n">
-        <v>-6</v>
+        <v>-3.53</v>
       </c>
       <c r="AJ4" s="3" t="n">
-        <v>955.8099999999999</v>
+        <v>13134.24</v>
       </c>
       <c r="AK4" s="3" t="n">
-        <v>12</v>
+        <v>14.94</v>
       </c>
       <c r="AL4" s="3" t="n">
-        <v>1058.22</v>
+        <v>14541.48</v>
       </c>
       <c r="AM4" s="3" t="n">
-        <v>24</v>
+        <v>27.26</v>
       </c>
       <c r="AN4" s="3" t="n">
-        <v>845</v>
+        <v>11600</v>
       </c>
       <c r="AO4" s="3" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="AP4" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="AQ4" s="3" t="inlineStr"/>
-      <c r="AR4" s="3" t="inlineStr"/>
+        <v>2.63</v>
+      </c>
+      <c r="AQ4" s="3" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="AR4" s="3" t="n">
+        <v>-3.08</v>
+      </c>
       <c r="AS4" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT4" s="3" t="inlineStr">
-        <is>
-          <t>Value · Mean Reversion · Ai Hybrid</t>
-        </is>
-      </c>
-      <c r="AU4" s="3" t="inlineStr"/>
+          <t>Quality · Growth · Momentum</t>
+        </is>
+      </c>
+      <c r="AT4" s="3" t="inlineStr"/>
+      <c r="AU4" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="AV4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="AW4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AX4" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW4" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ATUL_IND_20260806</t>
+          <t>INDIANB_IND_20260806</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1283,29 +1262,35 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>INDIANB</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>→ GNFC.NS · +7.4pp alpha</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>-0</v>
+      </c>
       <c r="K5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="L5" s="3" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="3" t="n">
-        <v>75.8</v>
+        <v>68.7</v>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
@@ -1318,7 +1303,7 @@
         </is>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>34.5</v>
+        <v>34.2</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>-0.8</v>
@@ -1330,12 +1315,12 @@
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-1.0%) · Rank #4 · Conf 35% · band HOLD · 17d left · → HOLD</t>
+          <t>🔴 AVOID · Rank #4 · Conf 35% · band HOLD · 17d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr"/>
       <c r="V5" s="3" t="n">
-        <v>35.2</v>
+        <v>35</v>
       </c>
       <c r="W5" s="3" t="inlineStr">
         <is>
@@ -1343,7 +1328,7 @@
         </is>
       </c>
       <c r="X5" s="3" t="n">
-        <v>25</v>
+        <v>25.4</v>
       </c>
       <c r="Y5" s="3" t="n">
         <v>1</v>
@@ -1363,64 +1348,59 @@
         </is>
       </c>
       <c r="AD5" s="3" t="n">
-        <v>6834</v>
+        <v>853.4</v>
       </c>
       <c r="AE5" s="3" t="n">
-        <v>6834</v>
+        <v>853.4000244140625</v>
       </c>
       <c r="AF5" s="3" t="n">
-        <v>6765.66</v>
+        <v>844.87</v>
       </c>
       <c r="AG5" s="3" t="n">
-        <v>6902.34</v>
+        <v>861.9299999999999</v>
       </c>
       <c r="AH5" s="3" t="n">
-        <v>6492.3</v>
+        <v>810.73</v>
       </c>
       <c r="AI5" s="3" t="n">
         <v>-5</v>
       </c>
       <c r="AJ5" s="3" t="n">
-        <v>7380.72</v>
+        <v>921.67</v>
       </c>
       <c r="AK5" s="3" t="n">
         <v>8</v>
       </c>
       <c r="AL5" s="3" t="n">
-        <v>7859.1</v>
+        <v>981.41</v>
       </c>
       <c r="AM5" s="3" t="n">
         <v>15</v>
       </c>
       <c r="AN5" s="3" t="n">
-        <v>6793.5</v>
+        <v>845</v>
       </c>
       <c r="AO5" s="3" t="n">
-        <v>0.6</v>
+        <v>0.99</v>
       </c>
       <c r="AP5" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AQ5" s="3" t="inlineStr"/>
       <c r="AR5" s="3" t="inlineStr"/>
       <c r="AS5" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT5" s="3" t="inlineStr">
-        <is>
-          <t>Trend · Growth · Mean Reversion</t>
-        </is>
-      </c>
+          <t>Value · Mean Reversion · Ai Hybrid</t>
+        </is>
+      </c>
+      <c r="AT5" s="3" t="inlineStr"/>
       <c r="AU5" s="3" t="inlineStr"/>
-      <c r="AV5" s="3" t="inlineStr"/>
-      <c r="AW5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX5" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV5" s="3" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="AW5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -1457,16 +1437,22 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>→ GNFC.NS · +7.8pp alpha</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0.35</v>
+      </c>
       <c r="K6" s="3" t="n">
         <v>5</v>
       </c>
@@ -1477,7 +1463,7 @@
         <v>-3</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>80.59999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
@@ -1502,7 +1488,7 @@
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-0.6%) · Rank ↑ 8→5 · Conf 43% · band STRONG · 16d left · → HOLD</t>
+          <t>🔴 AVOID · Rank ↑ 8→5 · Conf 43% · band STRONG · 16d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr"/>
@@ -1515,7 +1501,7 @@
         </is>
       </c>
       <c r="X6" s="3" t="n">
-        <v>24.8</v>
+        <v>25.1</v>
       </c>
       <c r="Y6" s="3" t="n">
         <v>2</v>
@@ -1581,29 +1567,24 @@
       </c>
       <c r="AS6" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT6" s="3" t="inlineStr">
-        <is>
-          <t>Trend · Quality · Mean Reversion</t>
-        </is>
-      </c>
+          <t>Quality · Trend · Mean Reversion</t>
+        </is>
+      </c>
+      <c r="AT6" s="3" t="inlineStr"/>
       <c r="AU6" s="3" t="inlineStr"/>
-      <c r="AV6" s="3" t="inlineStr"/>
-      <c r="AW6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV6" s="3" t="n">
+        <v>7.79</v>
+      </c>
+      <c r="AW6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GNFC_IND_20260806</t>
+          <t>ATUL_IND_20260806</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1618,34 +1599,40 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>R2_NEW</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>GNFC</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>→ GNFC.NS · +8.0pp alpha</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="K7" s="3" t="n">
         <v>6</v>
       </c>
       <c r="L7" s="3" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="3" t="n">
-        <v>77</v>
+        <v>75.8</v>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
@@ -1658,7 +1645,7 @@
         </is>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>38.6</v>
+        <v>34.5</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>-0.8</v>
@@ -1670,12 +1657,12 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>🟢 BUY (Δ-1.0%) · Rank #6 · Conf 39% · band HOLD · 60d left · → HOLD</t>
+          <t>🔴 AVOID · Rank #6 · Conf 35% · band HOLD · 17d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr"/>
       <c r="V7" s="3" t="n">
-        <v>39.3</v>
+        <v>35.2</v>
       </c>
       <c r="W7" s="3" t="inlineStr">
         <is>
@@ -1683,7 +1670,7 @@
         </is>
       </c>
       <c r="X7" s="3" t="n">
-        <v>24.3</v>
+        <v>24.9</v>
       </c>
       <c r="Y7" s="3" t="n">
         <v>1</v>
@@ -1692,10 +1679,10 @@
         <v>0</v>
       </c>
       <c r="AA7" s="3" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="AB7" s="3" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="AC7" s="3" t="inlineStr">
         <is>
@@ -1703,40 +1690,40 @@
         </is>
       </c>
       <c r="AD7" s="3" t="n">
-        <v>553.3</v>
+        <v>6834</v>
       </c>
       <c r="AE7" s="3" t="n">
-        <v>553.2999877929688</v>
+        <v>6834</v>
       </c>
       <c r="AF7" s="3" t="n">
-        <v>547.77</v>
+        <v>6765.66</v>
       </c>
       <c r="AG7" s="3" t="n">
-        <v>558.83</v>
+        <v>6902.34</v>
       </c>
       <c r="AH7" s="3" t="n">
-        <v>525.63</v>
+        <v>6492.3</v>
       </c>
       <c r="AI7" s="3" t="n">
         <v>-5</v>
       </c>
       <c r="AJ7" s="3" t="n">
-        <v>597.5599999999999</v>
+        <v>7380.72</v>
       </c>
       <c r="AK7" s="3" t="n">
         <v>8</v>
       </c>
       <c r="AL7" s="3" t="n">
-        <v>636.29</v>
+        <v>7859.1</v>
       </c>
       <c r="AM7" s="3" t="n">
         <v>15</v>
       </c>
       <c r="AN7" s="3" t="n">
-        <v>519.75</v>
+        <v>6793.5</v>
       </c>
       <c r="AO7" s="3" t="n">
-        <v>6.46</v>
+        <v>0.6</v>
       </c>
       <c r="AP7" s="3" t="n">
         <v>0</v>
@@ -1745,22 +1732,17 @@
       <c r="AR7" s="3" t="inlineStr"/>
       <c r="AS7" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT7" s="3" t="inlineStr">
-        <is>
-          <t>Value · Momentum · Ai Hybrid</t>
-        </is>
-      </c>
+          <t>Trend · Growth · Mean Reversion</t>
+        </is>
+      </c>
+      <c r="AT7" s="3" t="inlineStr"/>
       <c r="AU7" s="3" t="inlineStr"/>
-      <c r="AV7" s="3" t="inlineStr"/>
-      <c r="AW7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX7" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV7" s="3" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="AW7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1785,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +5.5pp alpha</t>
+          <t>→ GNFC.NS · +10.3pp alpha</t>
         </is>
       </c>
       <c r="J8" s="3" t="n">
@@ -1815,7 +1797,7 @@
       <c r="L8" s="3" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="3" t="n">
-        <v>63.4</v>
+        <v>63.1</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
@@ -1840,7 +1822,7 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank #7 · Conf 41% · band HOLD · 17d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank #7 · Conf 41% · band HOLD · 17d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr"/>
@@ -1853,7 +1835,7 @@
         </is>
       </c>
       <c r="X8" s="3" t="n">
-        <v>22.9</v>
+        <v>22.5</v>
       </c>
       <c r="Y8" s="3" t="n">
         <v>1</v>
@@ -1919,22 +1901,17 @@
       </c>
       <c r="AS8" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT8" s="3" t="inlineStr">
-        <is>
           <t>Mean Reversion · Value · Ai Hybrid</t>
         </is>
       </c>
+      <c r="AT8" s="3" t="inlineStr"/>
       <c r="AU8" s="3" t="inlineStr"/>
-      <c r="AV8" s="3" t="inlineStr"/>
-      <c r="AW8" s="3" t="n">
-        <v>5.47</v>
-      </c>
-      <c r="AX8" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV8" s="3" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="AW8" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1958,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +6.4pp alpha</t>
+          <t>→ GNFC.NS · +10.6pp alpha</t>
         </is>
       </c>
       <c r="J9" s="3" t="n">
@@ -2022,7 +1999,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank ↓ 2→8 · Conf 38% · band STRONG · 16d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank ↓ 2→8 · Conf 38% · band STRONG · 16d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr"/>
@@ -2035,7 +2012,7 @@
         </is>
       </c>
       <c r="X9" s="3" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="Y9" s="3" t="n">
         <v>2</v>
@@ -2101,22 +2078,17 @@
       </c>
       <c r="AS9" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT9" s="3" t="inlineStr">
-        <is>
           <t>Trend · Quality · Growth</t>
         </is>
       </c>
+      <c r="AT9" s="3" t="inlineStr"/>
       <c r="AU9" s="3" t="inlineStr"/>
-      <c r="AV9" s="3" t="inlineStr"/>
-      <c r="AW9" s="3" t="n">
-        <v>6.42</v>
-      </c>
-      <c r="AX9" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV9" s="3" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="AW9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2135,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +7.1pp alpha</t>
+          <t>→ GNFC.NS · +11.6pp alpha</t>
         </is>
       </c>
       <c r="J10" s="3" t="n">
@@ -2179,7 +2151,7 @@
         <v>3</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>64</v>
+        <v>63.9</v>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
@@ -2204,7 +2176,7 @@
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank ↓ 6→9 · Conf 33% · band HOLD · 60d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank ↓ 6→9 · Conf 33% · band HOLD · 17d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr"/>
@@ -2217,7 +2189,7 @@
         </is>
       </c>
       <c r="X10" s="3" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="Y10" s="3" t="n">
         <v>1</v>
@@ -2226,10 +2198,10 @@
         <v>6</v>
       </c>
       <c r="AA10" s="3" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="AB10" s="3" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="AC10" s="3" t="inlineStr">
         <is>
@@ -2283,29 +2255,24 @@
       </c>
       <c r="AS10" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT10" s="3" t="inlineStr">
-        <is>
           <t>Mean Reversion · Value · Growth</t>
         </is>
       </c>
+      <c r="AT10" s="3" t="inlineStr"/>
       <c r="AU10" s="3" t="inlineStr"/>
-      <c r="AV10" s="3" t="inlineStr"/>
-      <c r="AW10" s="3" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="AX10" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV10" s="3" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="AW10" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>NATIONALUM_IND_20260806</t>
+          <t>INFY_IND_20260730</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -2325,7 +2292,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>NATIONALUM</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
@@ -2341,19 +2308,23 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +7.3pp alpha</t>
+          <t>→ GNFC.NS · +11.7pp alpha</t>
         </is>
       </c>
       <c r="J11" s="3" t="n">
-        <v>-0</v>
+        <v>1.85</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="N11" s="3" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
@@ -2366,7 +2337,7 @@
         </is>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>39.9</v>
+        <v>40</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>-0.8</v>
@@ -2378,12 +2349,12 @@
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank #10 · Conf 41% · band HOLD · 17d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank ↓ 7→10 · Conf 41% · band HOLD · 59d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U11" s="3" t="inlineStr"/>
       <c r="V11" s="3" t="n">
-        <v>40.6</v>
+        <v>40.7</v>
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
@@ -2394,88 +2365,87 @@
         <v>21.1</v>
       </c>
       <c r="Y11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z11" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA11" s="3" t="n">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="AB11" s="3" t="n">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="AC11" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="AD11" s="3" t="n">
-        <v>380.35</v>
+        <v>1177</v>
       </c>
       <c r="AE11" s="3" t="n">
-        <v>380.3500061035156</v>
+        <v>1155.6</v>
       </c>
       <c r="AF11" s="3" t="n">
-        <v>376.55</v>
+        <v>1144.04</v>
       </c>
       <c r="AG11" s="3" t="n">
-        <v>384.15</v>
+        <v>1167.16</v>
       </c>
       <c r="AH11" s="3" t="n">
-        <v>361.33</v>
+        <v>1097.82</v>
       </c>
       <c r="AI11" s="3" t="n">
         <v>-5</v>
       </c>
       <c r="AJ11" s="3" t="n">
-        <v>410.78</v>
+        <v>1248.05</v>
       </c>
       <c r="AK11" s="3" t="n">
         <v>8</v>
       </c>
       <c r="AL11" s="3" t="n">
-        <v>437.4</v>
+        <v>1328.94</v>
       </c>
       <c r="AM11" s="3" t="n">
         <v>15</v>
       </c>
       <c r="AN11" s="3" t="n">
-        <v>377</v>
+        <v>1167.5</v>
       </c>
       <c r="AO11" s="3" t="n">
-        <v>0.89</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AP11" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="AQ11" s="3" t="inlineStr"/>
-      <c r="AR11" s="3" t="inlineStr"/>
+        <v>1.85</v>
+      </c>
+      <c r="AQ11" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AR11" s="3" t="n">
+        <v>-3.51</v>
+      </c>
       <c r="AS11" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT11" s="3" t="inlineStr">
-        <is>
-          <t>Mean Reversion · Quality · Value</t>
-        </is>
-      </c>
+          <t>Mean Reversion · Quality · Momentum</t>
+        </is>
+      </c>
+      <c r="AT11" s="3" t="inlineStr"/>
       <c r="AU11" s="3" t="inlineStr"/>
-      <c r="AV11" s="3" t="inlineStr"/>
-      <c r="AW11" s="3" t="n">
-        <v>7.31</v>
-      </c>
-      <c r="AX11" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV11" s="3" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="AW11" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AMBER_IND_20260729</t>
+          <t>BHARATFORG_IND_20260730</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2495,14 +2465,10 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>AMBER</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Amber Ent.</t>
-        </is>
-      </c>
+          <t>BHARATFORG</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr">
         <is>
           <t>EXIT</t>
@@ -2515,23 +2481,23 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +55.4pp alpha</t>
+          <t>→ GNFC.NS · +59.7pp alpha</t>
         </is>
       </c>
       <c r="J12" s="3" t="n">
-        <v>1.94</v>
+        <v>0.48</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>11</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>52.2</v>
+        <v>52.5</v>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
@@ -2544,7 +2510,7 @@
         </is>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>23.3</v>
+        <v>29.2</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>-0.8</v>
@@ -2556,12 +2522,12 @@
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank ↑ 14→11 · Conf 24% · band EXIT · 60d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank ↑ 13→11 · Conf 30% · band EXIT · 59d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U12" s="3" t="inlineStr"/>
       <c r="V12" s="3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="W12" s="3" t="inlineStr">
         <is>
@@ -2569,88 +2535,83 @@
         </is>
       </c>
       <c r="X12" s="3" t="n">
-        <v>-27</v>
+        <v>-26.9</v>
       </c>
       <c r="Y12" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z12" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA12" s="3" t="n">
         <v>60</v>
       </c>
       <c r="AB12" s="3" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AC12" s="3" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="AD12" s="3" t="n">
-        <v>7531.5</v>
+        <v>2182</v>
       </c>
       <c r="AE12" s="3" t="n">
-        <v>7388.5</v>
+        <v>2171.5</v>
       </c>
       <c r="AF12" s="3" t="n">
-        <v>7314.61</v>
+        <v>2149.78</v>
       </c>
       <c r="AG12" s="3" t="n">
-        <v>7462.39</v>
+        <v>2193.22</v>
       </c>
       <c r="AH12" s="3" t="n">
-        <v>7019.07</v>
+        <v>2062.92</v>
       </c>
       <c r="AI12" s="3" t="n">
         <v>-5</v>
       </c>
       <c r="AJ12" s="3" t="n">
-        <v>7979.58</v>
+        <v>2345.22</v>
       </c>
       <c r="AK12" s="3" t="n">
         <v>8</v>
       </c>
       <c r="AL12" s="3" t="n">
-        <v>8496.77</v>
+        <v>2497.22</v>
       </c>
       <c r="AM12" s="3" t="n">
         <v>15</v>
       </c>
       <c r="AN12" s="3" t="n">
-        <v>7395</v>
+        <v>2195</v>
       </c>
       <c r="AO12" s="3" t="n">
-        <v>1.85</v>
+        <v>-0.59</v>
       </c>
       <c r="AP12" s="3" t="n">
-        <v>1.94</v>
+        <v>0.48</v>
       </c>
       <c r="AQ12" s="3" t="n">
-        <v>0.31</v>
+        <v>2.22</v>
       </c>
       <c r="AR12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="AS12" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT12" s="3" t="inlineStr">
-        <is>
-          <t>Adx 14 · Atr 14 Pct · Distance From 52W High Pct · Distance From 52W Low Pct · Fund Debt To Equity</t>
-        </is>
-      </c>
+          <t>Adx 14 · Atr 14 Pct · Ca Days Since Last Dividend · Ca Last Dividend Amount · Distance From 52W High Pct</t>
+        </is>
+      </c>
+      <c r="AT12" s="3" t="inlineStr"/>
       <c r="AU12" s="3" t="inlineStr"/>
-      <c r="AV12" s="3" t="inlineStr"/>
-      <c r="AW12" s="3" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="AX12" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV12" s="3" t="n">
+        <v>59.69</v>
+      </c>
+      <c r="AW12" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2658,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +55.4pp alpha</t>
+          <t>→ GNFC.NS · +59.9pp alpha</t>
         </is>
       </c>
       <c r="J13" s="3" t="n">
@@ -2738,7 +2699,7 @@
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank ↓ 11→12 · Conf 30% · band EXIT · 16d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank ↓ 11→12 · Conf 30% · band EXIT · 16d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U13" s="3" t="inlineStr"/>
@@ -2751,7 +2712,7 @@
         </is>
       </c>
       <c r="X13" s="3" t="n">
-        <v>-27.1</v>
+        <v>-27</v>
       </c>
       <c r="Y13" s="3" t="n">
         <v>2</v>
@@ -2817,22 +2778,17 @@
       </c>
       <c r="AS13" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT13" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Ca Days Since Last Dividend · Ca Last Dividend Amount · Distance From 52W High Pct</t>
         </is>
       </c>
+      <c r="AT13" s="3" t="inlineStr"/>
       <c r="AU13" s="3" t="inlineStr"/>
-      <c r="AV13" s="3" t="inlineStr"/>
-      <c r="AW13" s="3" t="n">
-        <v>55.43</v>
-      </c>
-      <c r="AX13" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV13" s="3" t="n">
+        <v>59.88</v>
+      </c>
+      <c r="AW13" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2831,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +56.3pp alpha</t>
+          <t>→ GNFC.NS · +60.7pp alpha</t>
         </is>
       </c>
       <c r="J14" s="3" t="n">
@@ -2912,7 +2868,7 @@
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank #13 · Conf 25% · band EXIT · 60d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank #13 · Conf 25% · band EXIT · 17d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U14" s="3" t="inlineStr"/>
@@ -2925,7 +2881,7 @@
         </is>
       </c>
       <c r="X14" s="3" t="n">
-        <v>-28</v>
+        <v>-27.8</v>
       </c>
       <c r="Y14" s="3" t="n">
         <v>1</v>
@@ -2934,10 +2890,10 @@
         <v>0</v>
       </c>
       <c r="AA14" s="3" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="AB14" s="3" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="AC14" s="3" t="inlineStr">
         <is>
@@ -2987,22 +2943,17 @@
       <c r="AR14" s="3" t="inlineStr"/>
       <c r="AS14" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT14" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Distance From 52W High Pct · Distance From 52W Low Pct · Earn Days To Next</t>
         </is>
       </c>
+      <c r="AT14" s="3" t="inlineStr"/>
       <c r="AU14" s="3" t="inlineStr"/>
-      <c r="AV14" s="3" t="inlineStr"/>
-      <c r="AW14" s="3" t="n">
-        <v>56.33</v>
-      </c>
-      <c r="AX14" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV14" s="3" t="n">
+        <v>60.67</v>
+      </c>
+      <c r="AW14" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -3045,7 +2996,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +58.3pp alpha</t>
+          <t>→ GNFC.NS · +62.5pp alpha</t>
         </is>
       </c>
       <c r="J15" s="3" t="n">
@@ -3082,7 +3033,7 @@
       </c>
       <c r="T15" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank #14 · Conf 25% · band EXIT · 17d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank #14 · Conf 25% · band EXIT · 17d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U15" s="3" t="inlineStr"/>
@@ -3095,7 +3046,7 @@
         </is>
       </c>
       <c r="X15" s="3" t="n">
-        <v>-29.9</v>
+        <v>-29.7</v>
       </c>
       <c r="Y15" s="3" t="n">
         <v>1</v>
@@ -3157,22 +3108,17 @@
       <c r="AR15" s="3" t="inlineStr"/>
       <c r="AS15" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT15" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Distance From 52W High Pct · Distance From 52W Low Pct · Earn Days To Next</t>
         </is>
       </c>
+      <c r="AT15" s="3" t="inlineStr"/>
       <c r="AU15" s="3" t="inlineStr"/>
-      <c r="AV15" s="3" t="inlineStr"/>
-      <c r="AW15" s="3" t="n">
-        <v>58.32</v>
-      </c>
-      <c r="AX15" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV15" s="3" t="n">
+        <v>62.51</v>
+      </c>
+      <c r="AW15" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3161,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>→ TCS.NS · +60.5pp alpha</t>
+          <t>→ GNFC.NS · +64.8pp alpha</t>
         </is>
       </c>
       <c r="J16" s="3" t="n">
@@ -3252,7 +3198,7 @@
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>🔴 AVOID · Rank #15 · Conf 24% · band EXIT · 17d left · → EXIT (rotate to TCS.NS)</t>
+          <t>🔴 AVOID · Rank #15 · Conf 24% · band EXIT · 17d left · → EXIT (rotate to GNFC.NS)</t>
         </is>
       </c>
       <c r="U16" s="3" t="inlineStr"/>
@@ -3265,7 +3211,7 @@
         </is>
       </c>
       <c r="X16" s="3" t="n">
-        <v>-32.1</v>
+        <v>-32</v>
       </c>
       <c r="Y16" s="3" t="n">
         <v>1</v>
@@ -3331,22 +3277,17 @@
       </c>
       <c r="AS16" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT16" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Ca Days Since Last Dividend · Ca Last Dividend Amount · Distance From 52W High Pct</t>
         </is>
       </c>
+      <c r="AT16" s="3" t="inlineStr"/>
       <c r="AU16" s="3" t="inlineStr"/>
-      <c r="AV16" s="3" t="inlineStr"/>
-      <c r="AW16" s="3" t="n">
-        <v>60.46</v>
-      </c>
-      <c r="AX16" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AV16" s="3" t="n">
+        <v>64.81999999999999</v>
+      </c>
+      <c r="AW16" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -3481,26 +3422,21 @@
       </c>
       <c r="AQ17" s="3" t="inlineStr"/>
       <c r="AR17" s="3" t="inlineStr"/>
-      <c r="AS17" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT17" s="3" t="inlineStr"/>
-      <c r="AU17" s="3" t="inlineStr">
+      <c r="AS17" s="3" t="inlineStr"/>
+      <c r="AT17" s="3" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
+      <c r="AU17" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV17" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW17" s="3" t="n">
         <v>5.34</v>
       </c>
-      <c r="AX17" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -3635,26 +3571,21 @@
       </c>
       <c r="AQ18" s="3" t="inlineStr"/>
       <c r="AR18" s="3" t="inlineStr"/>
-      <c r="AS18" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT18" s="3" t="inlineStr"/>
-      <c r="AU18" s="3" t="inlineStr">
+      <c r="AS18" s="3" t="inlineStr"/>
+      <c r="AT18" s="3" t="inlineStr">
         <is>
           <t>Pharma</t>
         </is>
       </c>
+      <c r="AU18" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV18" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW18" s="3" t="n">
         <v>4.57</v>
       </c>
-      <c r="AX18" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW18" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -3793,26 +3724,21 @@
       <c r="AR19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS19" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT19" s="3" t="inlineStr"/>
-      <c r="AU19" s="3" t="inlineStr">
+      <c r="AS19" s="3" t="inlineStr"/>
+      <c r="AT19" s="3" t="inlineStr">
         <is>
           <t>Pharma</t>
         </is>
       </c>
+      <c r="AU19" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV19" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW19" s="3" t="n">
         <v>5.66</v>
       </c>
-      <c r="AX19" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW19" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -3947,26 +3873,21 @@
       </c>
       <c r="AQ20" s="3" t="inlineStr"/>
       <c r="AR20" s="3" t="inlineStr"/>
-      <c r="AS20" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT20" s="3" t="inlineStr"/>
-      <c r="AU20" s="3" t="inlineStr">
+      <c r="AS20" s="3" t="inlineStr"/>
+      <c r="AT20" s="3" t="inlineStr">
         <is>
           <t>Chemicals</t>
         </is>
       </c>
+      <c r="AU20" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV20" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW20" s="3" t="n">
         <v>1.39</v>
       </c>
-      <c r="AX20" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW20" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -4101,26 +4022,21 @@
       </c>
       <c r="AQ21" s="3" t="inlineStr"/>
       <c r="AR21" s="3" t="inlineStr"/>
-      <c r="AS21" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT21" s="3" t="inlineStr"/>
-      <c r="AU21" s="3" t="inlineStr">
+      <c r="AS21" s="3" t="inlineStr"/>
+      <c r="AT21" s="3" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
+      <c r="AU21" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV21" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW21" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX21" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW21" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -4255,26 +4171,21 @@
       </c>
       <c r="AQ22" s="3" t="inlineStr"/>
       <c r="AR22" s="3" t="inlineStr"/>
-      <c r="AS22" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT22" s="3" t="inlineStr"/>
-      <c r="AU22" s="3" t="inlineStr">
+      <c r="AS22" s="3" t="inlineStr"/>
+      <c r="AT22" s="3" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
+      <c r="AU22" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV22" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW22" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX22" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW22" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -4409,26 +4320,21 @@
       </c>
       <c r="AQ23" s="3" t="inlineStr"/>
       <c r="AR23" s="3" t="inlineStr"/>
-      <c r="AS23" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT23" s="3" t="inlineStr"/>
-      <c r="AU23" s="3" t="inlineStr">
+      <c r="AS23" s="3" t="inlineStr"/>
+      <c r="AT23" s="3" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
+      <c r="AU23" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV23" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW23" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX23" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW23" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -4563,26 +4469,21 @@
       <c r="AR24" s="3" t="n">
         <v>-1.5</v>
       </c>
-      <c r="AS24" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT24" s="3" t="inlineStr"/>
-      <c r="AU24" s="3" t="inlineStr">
+      <c r="AS24" s="3" t="inlineStr"/>
+      <c r="AT24" s="3" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
+      <c r="AU24" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV24" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW24" s="3" t="n">
         <v>-0.07000000000000001</v>
       </c>
-      <c r="AX24" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW24" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -4717,26 +4618,21 @@
       </c>
       <c r="AQ25" s="3" t="inlineStr"/>
       <c r="AR25" s="3" t="inlineStr"/>
-      <c r="AS25" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT25" s="3" t="inlineStr"/>
-      <c r="AU25" s="3" t="inlineStr">
+      <c r="AS25" s="3" t="inlineStr"/>
+      <c r="AT25" s="3" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
+      <c r="AU25" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV25" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW25" s="3" t="n">
         <v>8.01</v>
       </c>
-      <c r="AX25" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW25" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -4871,26 +4767,21 @@
       </c>
       <c r="AQ26" s="3" t="inlineStr"/>
       <c r="AR26" s="3" t="inlineStr"/>
-      <c r="AS26" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT26" s="3" t="inlineStr"/>
-      <c r="AU26" s="3" t="inlineStr">
+      <c r="AS26" s="3" t="inlineStr"/>
+      <c r="AT26" s="3" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
+      <c r="AU26" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV26" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW26" s="3" t="n">
         <v>7.99</v>
       </c>
-      <c r="AX26" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW26" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -5029,26 +4920,21 @@
       <c r="AR27" s="3" t="n">
         <v>-0.11</v>
       </c>
-      <c r="AS27" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT27" s="3" t="inlineStr"/>
-      <c r="AU27" s="3" t="inlineStr">
+      <c r="AS27" s="3" t="inlineStr"/>
+      <c r="AT27" s="3" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
+      <c r="AU27" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV27" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW27" s="3" t="n">
         <v>8.92</v>
       </c>
-      <c r="AX27" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW27" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -5179,26 +5065,21 @@
       </c>
       <c r="AQ28" s="3" t="inlineStr"/>
       <c r="AR28" s="3" t="inlineStr"/>
-      <c r="AS28" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT28" s="3" t="inlineStr"/>
-      <c r="AU28" s="3" t="inlineStr">
+      <c r="AS28" s="3" t="inlineStr"/>
+      <c r="AT28" s="3" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
+      <c r="AU28" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV28" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW28" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX28" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW28" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -5337,20 +5218,15 @@
       <c r="AR29" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS29" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS29" s="3" t="inlineStr"/>
       <c r="AT29" s="3" t="inlineStr"/>
       <c r="AU29" s="3" t="inlineStr"/>
-      <c r="AV29" s="3" t="inlineStr"/>
-      <c r="AW29" s="3" t="n">
+      <c r="AV29" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX29" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW29" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -5485,20 +5361,15 @@
       <c r="AR30" s="3" t="n">
         <v>-0.32</v>
       </c>
-      <c r="AS30" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS30" s="3" t="inlineStr"/>
       <c r="AT30" s="3" t="inlineStr"/>
       <c r="AU30" s="3" t="inlineStr"/>
-      <c r="AV30" s="3" t="inlineStr"/>
-      <c r="AW30" s="3" t="n">
+      <c r="AV30" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX30" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW30" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -5637,20 +5508,15 @@
       <c r="AR31" s="3" t="n">
         <v>-0.11</v>
       </c>
-      <c r="AS31" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS31" s="3" t="inlineStr"/>
       <c r="AT31" s="3" t="inlineStr"/>
       <c r="AU31" s="3" t="inlineStr"/>
-      <c r="AV31" s="3" t="inlineStr"/>
-      <c r="AW31" s="3" t="n">
+      <c r="AV31" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX31" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW31" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -5785,20 +5651,15 @@
       <c r="AR32" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS32" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS32" s="3" t="inlineStr"/>
       <c r="AT32" s="3" t="inlineStr"/>
       <c r="AU32" s="3" t="inlineStr"/>
-      <c r="AV32" s="3" t="inlineStr"/>
-      <c r="AW32" s="3" t="n">
+      <c r="AV32" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX32" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW32" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -5933,20 +5794,15 @@
       <c r="AR33" s="3" t="n">
         <v>-0.24</v>
       </c>
-      <c r="AS33" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS33" s="3" t="inlineStr"/>
       <c r="AT33" s="3" t="inlineStr"/>
       <c r="AU33" s="3" t="inlineStr"/>
-      <c r="AV33" s="3" t="inlineStr"/>
-      <c r="AW33" s="3" t="n">
+      <c r="AV33" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX33" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW33" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6047,18 +5903,13 @@
       <c r="AP34" s="3" t="inlineStr"/>
       <c r="AQ34" s="3" t="inlineStr"/>
       <c r="AR34" s="3" t="inlineStr"/>
-      <c r="AS34" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS34" s="3" t="inlineStr"/>
       <c r="AT34" s="3" t="inlineStr"/>
       <c r="AU34" s="3" t="inlineStr"/>
       <c r="AV34" s="3" t="inlineStr"/>
-      <c r="AW34" s="3" t="inlineStr"/>
-      <c r="AX34" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW34" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6159,18 +6010,13 @@
       <c r="AP35" s="3" t="inlineStr"/>
       <c r="AQ35" s="3" t="inlineStr"/>
       <c r="AR35" s="3" t="inlineStr"/>
-      <c r="AS35" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS35" s="3" t="inlineStr"/>
       <c r="AT35" s="3" t="inlineStr"/>
       <c r="AU35" s="3" t="inlineStr"/>
       <c r="AV35" s="3" t="inlineStr"/>
-      <c r="AW35" s="3" t="inlineStr"/>
-      <c r="AX35" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW35" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6279,18 +6125,13 @@
       <c r="AP36" s="3" t="inlineStr"/>
       <c r="AQ36" s="3" t="inlineStr"/>
       <c r="AR36" s="3" t="inlineStr"/>
-      <c r="AS36" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS36" s="3" t="inlineStr"/>
       <c r="AT36" s="3" t="inlineStr"/>
       <c r="AU36" s="3" t="inlineStr"/>
       <c r="AV36" s="3" t="inlineStr"/>
-      <c r="AW36" s="3" t="inlineStr"/>
-      <c r="AX36" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW36" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6399,18 +6240,13 @@
       <c r="AP37" s="3" t="inlineStr"/>
       <c r="AQ37" s="3" t="inlineStr"/>
       <c r="AR37" s="3" t="inlineStr"/>
-      <c r="AS37" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS37" s="3" t="inlineStr"/>
       <c r="AT37" s="3" t="inlineStr"/>
       <c r="AU37" s="3" t="inlineStr"/>
       <c r="AV37" s="3" t="inlineStr"/>
-      <c r="AW37" s="3" t="inlineStr"/>
-      <c r="AX37" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW37" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6549,20 +6385,15 @@
       <c r="AR38" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS38" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS38" s="3" t="inlineStr"/>
       <c r="AT38" s="3" t="inlineStr"/>
       <c r="AU38" s="3" t="inlineStr"/>
-      <c r="AV38" s="3" t="inlineStr"/>
-      <c r="AW38" s="3" t="n">
+      <c r="AV38" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX38" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW38" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6671,18 +6502,13 @@
       <c r="AP39" s="3" t="inlineStr"/>
       <c r="AQ39" s="3" t="inlineStr"/>
       <c r="AR39" s="3" t="inlineStr"/>
-      <c r="AS39" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS39" s="3" t="inlineStr"/>
       <c r="AT39" s="3" t="inlineStr"/>
       <c r="AU39" s="3" t="inlineStr"/>
       <c r="AV39" s="3" t="inlineStr"/>
-      <c r="AW39" s="3" t="inlineStr"/>
-      <c r="AX39" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW39" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6791,18 +6617,13 @@
       <c r="AP40" s="3" t="inlineStr"/>
       <c r="AQ40" s="3" t="inlineStr"/>
       <c r="AR40" s="3" t="inlineStr"/>
-      <c r="AS40" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS40" s="3" t="inlineStr"/>
       <c r="AT40" s="3" t="inlineStr"/>
       <c r="AU40" s="3" t="inlineStr"/>
       <c r="AV40" s="3" t="inlineStr"/>
-      <c r="AW40" s="3" t="inlineStr"/>
-      <c r="AX40" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW40" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -6911,18 +6732,13 @@
       <c r="AP41" s="3" t="inlineStr"/>
       <c r="AQ41" s="3" t="inlineStr"/>
       <c r="AR41" s="3" t="inlineStr"/>
-      <c r="AS41" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS41" s="3" t="inlineStr"/>
       <c r="AT41" s="3" t="inlineStr"/>
       <c r="AU41" s="3" t="inlineStr"/>
       <c r="AV41" s="3" t="inlineStr"/>
-      <c r="AW41" s="3" t="inlineStr"/>
-      <c r="AX41" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW41" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -7031,18 +6847,13 @@
       <c r="AP42" s="3" t="inlineStr"/>
       <c r="AQ42" s="3" t="inlineStr"/>
       <c r="AR42" s="3" t="inlineStr"/>
-      <c r="AS42" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS42" s="3" t="inlineStr"/>
       <c r="AT42" s="3" t="inlineStr"/>
       <c r="AU42" s="3" t="inlineStr"/>
       <c r="AV42" s="3" t="inlineStr"/>
-      <c r="AW42" s="3" t="inlineStr"/>
-      <c r="AX42" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW42" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -7151,18 +6962,13 @@
       <c r="AP43" s="3" t="inlineStr"/>
       <c r="AQ43" s="3" t="inlineStr"/>
       <c r="AR43" s="3" t="inlineStr"/>
-      <c r="AS43" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS43" s="3" t="inlineStr"/>
       <c r="AT43" s="3" t="inlineStr"/>
       <c r="AU43" s="3" t="inlineStr"/>
       <c r="AV43" s="3" t="inlineStr"/>
-      <c r="AW43" s="3" t="inlineStr"/>
-      <c r="AX43" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW43" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -7271,18 +7077,13 @@
       <c r="AP44" s="3" t="inlineStr"/>
       <c r="AQ44" s="3" t="inlineStr"/>
       <c r="AR44" s="3" t="inlineStr"/>
-      <c r="AS44" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS44" s="3" t="inlineStr"/>
       <c r="AT44" s="3" t="inlineStr"/>
       <c r="AU44" s="3" t="inlineStr"/>
       <c r="AV44" s="3" t="inlineStr"/>
-      <c r="AW44" s="3" t="inlineStr"/>
-      <c r="AX44" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW44" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -7421,20 +7222,15 @@
       <c r="AR45" s="3" t="n">
         <v>-0.11</v>
       </c>
-      <c r="AS45" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS45" s="3" t="inlineStr"/>
       <c r="AT45" s="3" t="inlineStr"/>
       <c r="AU45" s="3" t="inlineStr"/>
-      <c r="AV45" s="3" t="inlineStr"/>
-      <c r="AW45" s="3" t="n">
+      <c r="AV45" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="AX45" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW45" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -7539,18 +7335,13 @@
       <c r="AP46" s="3" t="inlineStr"/>
       <c r="AQ46" s="3" t="inlineStr"/>
       <c r="AR46" s="3" t="inlineStr"/>
-      <c r="AS46" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS46" s="3" t="inlineStr"/>
       <c r="AT46" s="3" t="inlineStr"/>
       <c r="AU46" s="3" t="inlineStr"/>
       <c r="AV46" s="3" t="inlineStr"/>
-      <c r="AW46" s="3" t="inlineStr"/>
-      <c r="AX46" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW46" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -7659,18 +7450,13 @@
       <c r="AP47" s="3" t="inlineStr"/>
       <c r="AQ47" s="3" t="inlineStr"/>
       <c r="AR47" s="3" t="inlineStr"/>
-      <c r="AS47" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="AS47" s="3" t="inlineStr"/>
       <c r="AT47" s="3" t="inlineStr"/>
       <c r="AU47" s="3" t="inlineStr"/>
       <c r="AV47" s="3" t="inlineStr"/>
-      <c r="AW47" s="3" t="inlineStr"/>
-      <c r="AX47" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW47" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7541,11 @@
           <t>🟢 BUY (Δ-1.0%) · Rank → 1→1 · Conf 57% · band HOLD · 14d left · → BUY</t>
         </is>
       </c>
-      <c r="U48" s="3" t="inlineStr"/>
+      <c r="U48" s="3" t="inlineStr">
+        <is>
+          <t>WARNING·STOP_LOSS_HIT·-5.2% ≤ -5% · exit</t>
+        </is>
+      </c>
       <c r="V48" s="3" t="n">
         <v>56.8</v>
       </c>
@@ -7831,24 +7621,19 @@
       </c>
       <c r="AS48" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT48" s="3" t="inlineStr">
-        <is>
           <t>Momentum · Value · Trend</t>
         </is>
       </c>
-      <c r="AU48" s="3" t="inlineStr"/>
+      <c r="AT48" s="3" t="inlineStr"/>
+      <c r="AU48" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="AV48" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="AW48" s="3" t="n">
         <v>6.23</v>
       </c>
-      <c r="AX48" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW48" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -8009,22 +7794,17 @@
       </c>
       <c r="AS49" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT49" s="3" t="inlineStr">
-        <is>
           <t>Momentum · Trend · Quality</t>
         </is>
       </c>
+      <c r="AT49" s="3" t="inlineStr"/>
       <c r="AU49" s="3" t="inlineStr"/>
-      <c r="AV49" s="3" t="inlineStr"/>
-      <c r="AW49" s="3" t="n">
+      <c r="AV49" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AX49" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW49" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -8191,22 +7971,17 @@
       </c>
       <c r="AS50" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT50" s="3" t="inlineStr">
-        <is>
           <t>Quality · Growth · Mean Reversion</t>
         </is>
       </c>
+      <c r="AT50" s="3" t="inlineStr"/>
       <c r="AU50" s="3" t="inlineStr"/>
-      <c r="AV50" s="3" t="inlineStr"/>
-      <c r="AW50" s="3" t="n">
+      <c r="AV50" s="3" t="n">
         <v>12.15</v>
       </c>
-      <c r="AX50" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW50" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -8373,22 +8148,17 @@
       </c>
       <c r="AS51" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT51" s="3" t="inlineStr">
-        <is>
           <t>Momentum · Value · Mean Reversion</t>
         </is>
       </c>
+      <c r="AT51" s="3" t="inlineStr"/>
       <c r="AU51" s="3" t="inlineStr"/>
-      <c r="AV51" s="3" t="inlineStr"/>
-      <c r="AW51" s="3" t="n">
+      <c r="AV51" s="3" t="n">
         <v>12.97</v>
       </c>
-      <c r="AX51" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW51" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -8479,7 +8249,11 @@
           <t>🔴 AVOID · Rank → 5→5 · Conf 50% · band HOLD · 6d left · → EXIT (rotate to TRV)</t>
         </is>
       </c>
-      <c r="U52" s="3" t="inlineStr"/>
+      <c r="U52" s="3" t="inlineStr">
+        <is>
+          <t>WARNING·STOP_LOSS_HIT·-6.7% ≤ -5% · exit</t>
+        </is>
+      </c>
       <c r="V52" s="3" t="n">
         <v>50.5</v>
       </c>
@@ -8555,22 +8329,17 @@
       </c>
       <c r="AS52" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT52" s="3" t="inlineStr">
-        <is>
           <t>Mean Reversion · Growth · Value</t>
         </is>
       </c>
+      <c r="AT52" s="3" t="inlineStr"/>
       <c r="AU52" s="3" t="inlineStr"/>
-      <c r="AV52" s="3" t="inlineStr"/>
-      <c r="AW52" s="3" t="n">
+      <c r="AV52" s="3" t="n">
         <v>14.45</v>
       </c>
-      <c r="AX52" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW52" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -8737,22 +8506,17 @@
       </c>
       <c r="AS53" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT53" s="3" t="inlineStr">
-        <is>
           <t>Value · News · Event Driven</t>
         </is>
       </c>
+      <c r="AT53" s="3" t="inlineStr"/>
       <c r="AU53" s="3" t="inlineStr"/>
-      <c r="AV53" s="3" t="inlineStr"/>
-      <c r="AW53" s="3" t="n">
+      <c r="AV53" s="3" t="n">
         <v>14.77</v>
       </c>
-      <c r="AX53" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW53" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -8919,22 +8683,17 @@
       </c>
       <c r="AS54" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT54" s="3" t="inlineStr">
-        <is>
           <t>Value · Trend · Momentum</t>
         </is>
       </c>
+      <c r="AT54" s="3" t="inlineStr"/>
       <c r="AU54" s="3" t="inlineStr"/>
-      <c r="AV54" s="3" t="inlineStr"/>
-      <c r="AW54" s="3" t="n">
+      <c r="AV54" s="3" t="n">
         <v>14.87</v>
       </c>
-      <c r="AX54" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW54" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -9025,7 +8784,11 @@
           <t>🔴 AVOID · Rank → 8→8 · Conf 54% · band HOLD · 58d left · → EXIT (rotate to TRV)</t>
         </is>
       </c>
-      <c r="U55" s="3" t="inlineStr"/>
+      <c r="U55" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-12.7% ≤ -8% · EXIT URGENT</t>
+        </is>
+      </c>
       <c r="V55" s="3" t="n">
         <v>53.6</v>
       </c>
@@ -9101,22 +8864,17 @@
       </c>
       <c r="AS55" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT55" s="3" t="inlineStr">
-        <is>
           <t>Quality · Mean Reversion · Trend</t>
         </is>
       </c>
+      <c r="AT55" s="3" t="inlineStr"/>
       <c r="AU55" s="3" t="inlineStr"/>
-      <c r="AV55" s="3" t="inlineStr"/>
-      <c r="AW55" s="3" t="n">
+      <c r="AV55" s="3" t="n">
         <v>15.21</v>
       </c>
-      <c r="AX55" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW55" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -9207,7 +8965,11 @@
           <t>🔴 AVOID · Rank → 9→9 · Conf 50% · band STRONG · 6d left · → EXIT (rotate to TRV)</t>
         </is>
       </c>
-      <c r="U56" s="3" t="inlineStr"/>
+      <c r="U56" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-8.4% ≤ -8% · EXIT URGENT</t>
+        </is>
+      </c>
       <c r="V56" s="3" t="n">
         <v>50.5</v>
       </c>
@@ -9283,22 +9045,17 @@
       </c>
       <c r="AS56" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT56" s="3" t="inlineStr">
-        <is>
           <t>Momentum · News · Quality</t>
         </is>
       </c>
+      <c r="AT56" s="3" t="inlineStr"/>
       <c r="AU56" s="3" t="inlineStr"/>
-      <c r="AV56" s="3" t="inlineStr"/>
-      <c r="AW56" s="3" t="n">
+      <c r="AV56" s="3" t="n">
         <v>15.5</v>
       </c>
-      <c r="AX56" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW56" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -9389,7 +9146,11 @@
           <t>🔴 AVOID · Rank → 10→10 · Conf 54% · band HOLD · 58d left · → EXIT (rotate to TRV)</t>
         </is>
       </c>
-      <c r="U57" s="3" t="inlineStr"/>
+      <c r="U57" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-9.2% ≤ -8% · EXIT URGENT</t>
+        </is>
+      </c>
       <c r="V57" s="3" t="n">
         <v>53.6</v>
       </c>
@@ -9465,22 +9226,17 @@
       </c>
       <c r="AS57" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT57" s="3" t="inlineStr">
-        <is>
           <t>Momentum · News · Value</t>
         </is>
       </c>
+      <c r="AT57" s="3" t="inlineStr"/>
       <c r="AU57" s="3" t="inlineStr"/>
-      <c r="AV57" s="3" t="inlineStr"/>
-      <c r="AW57" s="3" t="n">
+      <c r="AV57" s="3" t="n">
         <v>16.4</v>
       </c>
-      <c r="AX57" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW57" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -9571,7 +9327,11 @@
           <t>🔴 AVOID · Rank → 11→11 · Conf 29% · band EXIT · 6d left · → EXIT (rotate to TRV)</t>
         </is>
       </c>
-      <c r="U58" s="3" t="inlineStr"/>
+      <c r="U58" s="3" t="inlineStr">
+        <is>
+          <t>WARNING·RAPID_APPRECIATION·+16.1% ≥ +12% · take profit</t>
+        </is>
+      </c>
       <c r="V58" s="3" t="n">
         <v>28.7</v>
       </c>
@@ -9647,22 +9407,17 @@
       </c>
       <c r="AS58" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT58" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Close · Distance From 52W High Pct · Distance From 52W Low Pct</t>
         </is>
       </c>
+      <c r="AT58" s="3" t="inlineStr"/>
       <c r="AU58" s="3" t="inlineStr"/>
-      <c r="AV58" s="3" t="inlineStr"/>
-      <c r="AW58" s="3" t="n">
+      <c r="AV58" s="3" t="n">
         <v>37.17</v>
       </c>
-      <c r="AX58" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW58" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -9829,22 +9584,17 @@
       </c>
       <c r="AS59" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT59" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Close · Distance From 52W High Pct · Distance From 52W Low Pct</t>
         </is>
       </c>
+      <c r="AT59" s="3" t="inlineStr"/>
       <c r="AU59" s="3" t="inlineStr"/>
-      <c r="AV59" s="3" t="inlineStr"/>
-      <c r="AW59" s="3" t="n">
+      <c r="AV59" s="3" t="n">
         <v>37.79</v>
       </c>
-      <c r="AX59" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW59" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -10011,22 +9761,17 @@
       </c>
       <c r="AS60" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT60" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Ca Days Since Last Dividend · Ca Last Dividend Amount · Close</t>
         </is>
       </c>
+      <c r="AT60" s="3" t="inlineStr"/>
       <c r="AU60" s="3" t="inlineStr"/>
-      <c r="AV60" s="3" t="inlineStr"/>
-      <c r="AW60" s="3" t="n">
+      <c r="AV60" s="3" t="n">
         <v>43.85</v>
       </c>
-      <c r="AX60" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW60" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -10193,22 +9938,17 @@
       </c>
       <c r="AS61" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT61" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Ca Days Since Last Dividend · Ca Last Dividend Amount · Close</t>
         </is>
       </c>
+      <c r="AT61" s="3" t="inlineStr"/>
       <c r="AU61" s="3" t="inlineStr"/>
-      <c r="AV61" s="3" t="inlineStr"/>
-      <c r="AW61" s="3" t="n">
+      <c r="AV61" s="3" t="n">
         <v>45.62</v>
       </c>
-      <c r="AX61" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW61" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -10375,22 +10115,17 @@
       </c>
       <c r="AS62" s="3" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT62" s="3" t="inlineStr">
-        <is>
           <t>Adx 14 · Atr 14 Pct · Ca Days Since Last Dividend · Ca Last Dividend Amount · Close</t>
         </is>
       </c>
+      <c r="AT62" s="3" t="inlineStr"/>
       <c r="AU62" s="3" t="inlineStr"/>
-      <c r="AV62" s="3" t="inlineStr"/>
-      <c r="AW62" s="3" t="n">
+      <c r="AV62" s="3" t="n">
         <v>45.94</v>
       </c>
-      <c r="AX62" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW62" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -10543,26 +10278,21 @@
       <c r="AR63" s="3" t="n">
         <v>-0.71</v>
       </c>
-      <c r="AS63" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT63" s="3" t="inlineStr"/>
-      <c r="AU63" s="3" t="inlineStr">
+      <c r="AS63" s="3" t="inlineStr"/>
+      <c r="AT63" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU63" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV63" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW63" s="3" t="n">
         <v>5.02</v>
       </c>
-      <c r="AX63" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW63" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -10643,7 +10373,11 @@
           <t>🟢 BUY (Δ-1.0%) · Rank #2 · Conf 57% · momentum → · band HOLD · 91d left · → BUY</t>
         </is>
       </c>
-      <c r="U64" s="3" t="inlineStr"/>
+      <c r="U64" s="3" t="inlineStr">
+        <is>
+          <t>WARNING·STOP_LOSS_HIT·-5.2% ≤ -5% · exit</t>
+        </is>
+      </c>
       <c r="V64" s="3" t="n">
         <v>56.8</v>
       </c>
@@ -10715,26 +10449,21 @@
       <c r="AR64" s="3" t="n">
         <v>-3.77</v>
       </c>
-      <c r="AS64" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT64" s="3" t="inlineStr"/>
-      <c r="AU64" s="3" t="inlineStr">
+      <c r="AS64" s="3" t="inlineStr"/>
+      <c r="AT64" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU64" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV64" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW64" s="3" t="n">
         <v>6.23</v>
       </c>
-      <c r="AX64" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW64" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -10887,26 +10616,21 @@
       <c r="AR65" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS65" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT65" s="3" t="inlineStr"/>
-      <c r="AU65" s="3" t="inlineStr">
+      <c r="AS65" s="3" t="inlineStr"/>
+      <c r="AT65" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU65" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV65" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW65" s="3" t="n">
         <v>15.28</v>
       </c>
-      <c r="AX65" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW65" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -10987,7 +10711,11 @@
           <t>🟢 BUY (Δ-2.0%) · Rank #4 · Conf 54% · momentum → · band HOLD · 91d left · → BUY</t>
         </is>
       </c>
-      <c r="U66" s="3" t="inlineStr"/>
+      <c r="U66" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-12.7% ≤ -8% · EXIT URGENT</t>
+        </is>
+      </c>
       <c r="V66" s="3" t="n">
         <v>53.6</v>
       </c>
@@ -11059,26 +10787,21 @@
       <c r="AR66" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS66" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT66" s="3" t="inlineStr"/>
-      <c r="AU66" s="3" t="inlineStr">
+      <c r="AS66" s="3" t="inlineStr"/>
+      <c r="AT66" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU66" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV66" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW66" s="3" t="n">
         <v>-5.71</v>
       </c>
-      <c r="AX66" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW66" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -11159,7 +10882,11 @@
           <t>🟢 BUY (Δ-2.0%) · Rank #5 · Conf 50% · momentum → · band STRONG · 91d left · → HOLD</t>
         </is>
       </c>
-      <c r="U67" s="3" t="inlineStr"/>
+      <c r="U67" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-8.4% ≤ -8% · EXIT URGENT</t>
+        </is>
+      </c>
       <c r="V67" s="3" t="n">
         <v>50.5</v>
       </c>
@@ -11231,26 +10958,21 @@
       <c r="AR67" s="3" t="n">
         <v>-1.67</v>
       </c>
-      <c r="AS67" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT67" s="3" t="inlineStr"/>
-      <c r="AU67" s="3" t="inlineStr">
+      <c r="AS67" s="3" t="inlineStr"/>
+      <c r="AT67" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU67" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV67" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW67" s="3" t="n">
         <v>-1.12</v>
       </c>
-      <c r="AX67" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW67" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -11331,7 +11053,11 @@
           <t>🟢 BUY (Δ-2.0%) · Rank #6 · Conf 50% · momentum → · band HOLD · 91d left · → HOLD</t>
         </is>
       </c>
-      <c r="U68" s="3" t="inlineStr"/>
+      <c r="U68" s="3" t="inlineStr">
+        <is>
+          <t>WARNING·STOP_LOSS_HIT·-6.7% ≤ -5% · exit</t>
+        </is>
+      </c>
       <c r="V68" s="3" t="n">
         <v>50.5</v>
       </c>
@@ -11403,26 +11129,21 @@
       <c r="AR68" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS68" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT68" s="3" t="inlineStr"/>
-      <c r="AU68" s="3" t="inlineStr">
+      <c r="AS68" s="3" t="inlineStr"/>
+      <c r="AT68" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU68" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV68" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW68" s="3" t="n">
         <v>0.79</v>
       </c>
-      <c r="AX68" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW68" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -11575,26 +11296,21 @@
       <c r="AR69" s="3" t="n">
         <v>-8.66</v>
       </c>
-      <c r="AS69" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT69" s="3" t="inlineStr"/>
-      <c r="AU69" s="3" t="inlineStr">
+      <c r="AS69" s="3" t="inlineStr"/>
+      <c r="AT69" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU69" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV69" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW69" s="3" t="n">
         <v>6.58</v>
       </c>
-      <c r="AX69" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW69" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -11747,26 +11463,21 @@
       <c r="AR70" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS70" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT70" s="3" t="inlineStr"/>
-      <c r="AU70" s="3" t="inlineStr">
+      <c r="AS70" s="3" t="inlineStr"/>
+      <c r="AT70" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU70" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV70" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW70" s="3" t="n">
         <v>6.87</v>
       </c>
-      <c r="AX70" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW70" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -11919,26 +11630,21 @@
       <c r="AR71" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS71" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT71" s="3" t="inlineStr"/>
-      <c r="AU71" s="3" t="inlineStr">
+      <c r="AS71" s="3" t="inlineStr"/>
+      <c r="AT71" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU71" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV71" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW71" s="3" t="n">
         <v>17.3</v>
       </c>
-      <c r="AX71" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW71" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
@@ -12019,7 +11725,11 @@
           <t>🟢 BUY (Δ-2.0%) · Rank #10 · Conf 54% · momentum → · band HOLD · 91d left · → HOLD</t>
         </is>
       </c>
-      <c r="U72" s="3" t="inlineStr"/>
+      <c r="U72" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL·DEEP_LOSS·-9.2% ≤ -8% · EXIT URGENT</t>
+        </is>
+      </c>
       <c r="V72" s="3" t="n">
         <v>53.6</v>
       </c>
@@ -12091,31 +11801,26 @@
       <c r="AR72" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AS72" s="3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="AT72" s="3" t="inlineStr"/>
-      <c r="AU72" s="3" t="inlineStr">
+      <c r="AS72" s="3" t="inlineStr"/>
+      <c r="AT72" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="AU72" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AV72" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AW72" s="3" t="n">
         <v>-1.96</v>
       </c>
-      <c r="AX72" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06 15:51</t>
+      <c r="AW72" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 04:01</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AX72"/>
+  <autoFilter ref="A1:AW72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>